<commit_message>
显式区分透明色 RGBA 数据：2026-05-19 17:41:44 CST
- 普通非透明颜色继续保持 #RRGGBB 和 [r,g,b]
- 透明颜色改为 #RRGGBBAA 和 [r,g,b,a]，并保留 transparency 字段
- CT01-CT09 使用 alpha 128，MH1 使用 alpha 0，避免数据消费者误当普通 RGB
- 生成器支持 6/8 位 HEX 与 3/4 通道 RGB，并能从 8 位 HEX 补 alpha
- XLSX 透明色块使用交错底纹，PDF 图例透明色使用棋盘格预览
- 更新 README/AGENTS 说明透明色口径并重生成交付物
</commit_message>
<xml_diff>
--- a/artkal-c-197-official/colors.xlsx
+++ b/artkal-c-197-official/colors.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="信息" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="01_C" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="02_CE" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="03_CG" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="04_CP" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="05_CT" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="信息" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_C" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_CE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_CG" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_CP" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_CT" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -55,7 +55,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="199">
+  <fills count="200">
     <fill>
       <patternFill/>
     </fill>
@@ -1004,47 +1004,52 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6C6D2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE664A6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF6875C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC4C764"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF32B195"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF757DD1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF4EB1DC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF5688A0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF6B849D"/>
+        <fgColor rgb="FFE2E2E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE0E0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2B1D2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFAC3AD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE1E3B1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF98D8CA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBABEE8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA6D8ED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFAAC3CF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB5C1CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -1074,7 +1079,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="402">
+  <cellXfs count="400">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1842,12 +1847,9 @@
     <xf numFmtId="0" fontId="5" fillId="190" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="191" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="190" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="191" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="191" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="192" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="191" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="192" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1855,26 +1857,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="193" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="194" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="194" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="195" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="195" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="196" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="196" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="197" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="197" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="198" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="198" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="198" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="199" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="199" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -10642,55 +10639,55 @@
         </is>
       </c>
       <c r="B4" s="385" t="n"/>
-      <c r="C4" s="385" t="n"/>
+      <c r="C4" s="386" t="n"/>
       <c r="D4" s="385" t="n"/>
-      <c r="F4" s="386" t="inlineStr">
+      <c r="F4" s="387" t="inlineStr">
         <is>
           <t>CT02</t>
         </is>
       </c>
-      <c r="G4" s="387" t="n"/>
-      <c r="H4" s="387" t="n"/>
-      <c r="I4" s="387" t="n"/>
-      <c r="K4" s="388" t="inlineStr">
+      <c r="G4" s="388" t="n"/>
+      <c r="H4" s="385" t="n"/>
+      <c r="I4" s="388" t="n"/>
+      <c r="K4" s="389" t="inlineStr">
         <is>
           <t>CT03</t>
         </is>
       </c>
-      <c r="L4" s="389" t="n"/>
-      <c r="M4" s="389" t="n"/>
-      <c r="N4" s="389" t="n"/>
-      <c r="P4" s="390" t="inlineStr">
+      <c r="L4" s="385" t="n"/>
+      <c r="M4" s="390" t="n"/>
+      <c r="N4" s="385" t="n"/>
+      <c r="P4" s="387" t="inlineStr">
         <is>
           <t>CT04</t>
         </is>
       </c>
       <c r="Q4" s="391" t="n"/>
-      <c r="R4" s="391" t="n"/>
+      <c r="R4" s="385" t="n"/>
       <c r="S4" s="391" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="385" t="n"/>
-      <c r="B5" s="385" t="n"/>
+      <c r="B5" s="386" t="n"/>
       <c r="C5" s="385" t="n"/>
-      <c r="D5" s="385" t="n"/>
-      <c r="F5" s="387" t="n"/>
-      <c r="G5" s="387" t="n"/>
-      <c r="H5" s="387" t="n"/>
-      <c r="I5" s="387" t="n"/>
-      <c r="K5" s="389" t="n"/>
-      <c r="L5" s="389" t="n"/>
-      <c r="M5" s="389" t="n"/>
-      <c r="N5" s="389" t="n"/>
+      <c r="D5" s="386" t="n"/>
+      <c r="F5" s="388" t="n"/>
+      <c r="G5" s="385" t="n"/>
+      <c r="H5" s="388" t="n"/>
+      <c r="I5" s="385" t="n"/>
+      <c r="K5" s="385" t="n"/>
+      <c r="L5" s="390" t="n"/>
+      <c r="M5" s="385" t="n"/>
+      <c r="N5" s="390" t="n"/>
       <c r="P5" s="391" t="n"/>
-      <c r="Q5" s="391" t="n"/>
+      <c r="Q5" s="385" t="n"/>
       <c r="R5" s="391" t="n"/>
-      <c r="S5" s="391" t="n"/>
+      <c r="S5" s="385" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>HEX: #C6C6D2</t>
+          <t>HEX: #C6C6D280</t>
         </is>
       </c>
       <c r="B6" s="15" t="n"/>
@@ -10698,7 +10695,7 @@
       <c r="D6" s="15" t="n"/>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>HEX: #E664A6</t>
+          <t>HEX: #E664A680</t>
         </is>
       </c>
       <c r="G6" s="15" t="n"/>
@@ -10706,7 +10703,7 @@
       <c r="I6" s="15" t="n"/>
       <c r="K6" s="14" t="inlineStr">
         <is>
-          <t>HEX: #F6875C</t>
+          <t>HEX: #F6875C80</t>
         </is>
       </c>
       <c r="L6" s="15" t="n"/>
@@ -10714,7 +10711,7 @@
       <c r="N6" s="15" t="n"/>
       <c r="P6" s="14" t="inlineStr">
         <is>
-          <t>HEX: #C4C764</t>
+          <t>HEX: #C4C76480</t>
         </is>
       </c>
       <c r="Q6" s="15" t="n"/>
@@ -10724,7 +10721,7 @@
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>RGB: 198, 198, 210</t>
+          <t>RGB: 198, 198, 210, 128</t>
         </is>
       </c>
       <c r="B7" s="15" t="n"/>
@@ -10732,7 +10729,7 @@
       <c r="D7" s="15" t="n"/>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>RGB: 230, 100, 166</t>
+          <t>RGB: 230, 100, 166, 128</t>
         </is>
       </c>
       <c r="G7" s="15" t="n"/>
@@ -10740,7 +10737,7 @@
       <c r="I7" s="15" t="n"/>
       <c r="K7" s="14" t="inlineStr">
         <is>
-          <t>RGB: 246, 135, 92</t>
+          <t>RGB: 246, 135, 92, 128</t>
         </is>
       </c>
       <c r="L7" s="15" t="n"/>
@@ -10748,7 +10745,7 @@
       <c r="N7" s="15" t="n"/>
       <c r="P7" s="14" t="inlineStr">
         <is>
-          <t>RGB: 196, 199, 100</t>
+          <t>RGB: 196, 199, 100, 128</t>
         </is>
       </c>
       <c r="Q7" s="15" t="n"/>
@@ -10790,61 +10787,61 @@
       <c r="S8" s="15" t="n"/>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="392" t="inlineStr">
+      <c r="A9" s="387" t="inlineStr">
         <is>
           <t>CT05</t>
         </is>
       </c>
-      <c r="B9" s="393" t="n"/>
-      <c r="C9" s="393" t="n"/>
-      <c r="D9" s="393" t="n"/>
-      <c r="F9" s="394" t="inlineStr">
+      <c r="B9" s="392" t="n"/>
+      <c r="C9" s="385" t="n"/>
+      <c r="D9" s="392" t="n"/>
+      <c r="F9" s="393" t="inlineStr">
         <is>
           <t>CT06</t>
         </is>
       </c>
-      <c r="G9" s="395" t="n"/>
-      <c r="H9" s="395" t="n"/>
-      <c r="I9" s="395" t="n"/>
-      <c r="K9" s="396" t="inlineStr">
+      <c r="G9" s="385" t="n"/>
+      <c r="H9" s="394" t="n"/>
+      <c r="I9" s="385" t="n"/>
+      <c r="K9" s="387" t="inlineStr">
         <is>
           <t>CT07</t>
         </is>
       </c>
-      <c r="L9" s="397" t="n"/>
-      <c r="M9" s="397" t="n"/>
-      <c r="N9" s="397" t="n"/>
-      <c r="P9" s="398" t="inlineStr">
+      <c r="L9" s="395" t="n"/>
+      <c r="M9" s="385" t="n"/>
+      <c r="N9" s="395" t="n"/>
+      <c r="P9" s="396" t="inlineStr">
         <is>
           <t>CT08</t>
         </is>
       </c>
-      <c r="Q9" s="399" t="n"/>
-      <c r="R9" s="399" t="n"/>
-      <c r="S9" s="399" t="n"/>
+      <c r="Q9" s="385" t="n"/>
+      <c r="R9" s="397" t="n"/>
+      <c r="S9" s="385" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="393" t="n"/>
-      <c r="B10" s="393" t="n"/>
-      <c r="C10" s="393" t="n"/>
-      <c r="D10" s="393" t="n"/>
-      <c r="F10" s="395" t="n"/>
-      <c r="G10" s="395" t="n"/>
-      <c r="H10" s="395" t="n"/>
-      <c r="I10" s="395" t="n"/>
-      <c r="K10" s="397" t="n"/>
-      <c r="L10" s="397" t="n"/>
-      <c r="M10" s="397" t="n"/>
-      <c r="N10" s="397" t="n"/>
-      <c r="P10" s="399" t="n"/>
-      <c r="Q10" s="399" t="n"/>
-      <c r="R10" s="399" t="n"/>
-      <c r="S10" s="399" t="n"/>
+      <c r="A10" s="392" t="n"/>
+      <c r="B10" s="385" t="n"/>
+      <c r="C10" s="392" t="n"/>
+      <c r="D10" s="385" t="n"/>
+      <c r="F10" s="385" t="n"/>
+      <c r="G10" s="394" t="n"/>
+      <c r="H10" s="385" t="n"/>
+      <c r="I10" s="394" t="n"/>
+      <c r="K10" s="395" t="n"/>
+      <c r="L10" s="385" t="n"/>
+      <c r="M10" s="395" t="n"/>
+      <c r="N10" s="385" t="n"/>
+      <c r="P10" s="385" t="n"/>
+      <c r="Q10" s="397" t="n"/>
+      <c r="R10" s="385" t="n"/>
+      <c r="S10" s="397" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>HEX: #32B195</t>
+          <t>HEX: #32B19580</t>
         </is>
       </c>
       <c r="B11" s="15" t="n"/>
@@ -10852,7 +10849,7 @@
       <c r="D11" s="15" t="n"/>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>HEX: #757DD1</t>
+          <t>HEX: #757DD180</t>
         </is>
       </c>
       <c r="G11" s="15" t="n"/>
@@ -10860,7 +10857,7 @@
       <c r="I11" s="15" t="n"/>
       <c r="K11" s="14" t="inlineStr">
         <is>
-          <t>HEX: #4EB1DC</t>
+          <t>HEX: #4EB1DC80</t>
         </is>
       </c>
       <c r="L11" s="15" t="n"/>
@@ -10868,7 +10865,7 @@
       <c r="N11" s="15" t="n"/>
       <c r="P11" s="14" t="inlineStr">
         <is>
-          <t>HEX: #5688A0</t>
+          <t>HEX: #5688A080</t>
         </is>
       </c>
       <c r="Q11" s="15" t="n"/>
@@ -10878,7 +10875,7 @@
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>RGB: 50, 177, 149</t>
+          <t>RGB: 50, 177, 149, 128</t>
         </is>
       </c>
       <c r="B12" s="15" t="n"/>
@@ -10886,7 +10883,7 @@
       <c r="D12" s="15" t="n"/>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>RGB: 117, 125, 209</t>
+          <t>RGB: 117, 125, 209, 128</t>
         </is>
       </c>
       <c r="G12" s="15" t="n"/>
@@ -10894,7 +10891,7 @@
       <c r="I12" s="15" t="n"/>
       <c r="K12" s="14" t="inlineStr">
         <is>
-          <t>RGB: 78, 177, 220</t>
+          <t>RGB: 78, 177, 220, 128</t>
         </is>
       </c>
       <c r="L12" s="15" t="n"/>
@@ -10902,7 +10899,7 @@
       <c r="N12" s="15" t="n"/>
       <c r="P12" s="14" t="inlineStr">
         <is>
-          <t>RGB: 86, 136, 160</t>
+          <t>RGB: 86, 136, 160, 128</t>
         </is>
       </c>
       <c r="Q12" s="15" t="n"/>
@@ -10944,25 +10941,25 @@
       <c r="S13" s="15" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="400" t="inlineStr">
+      <c r="A14" s="398" t="inlineStr">
         <is>
           <t>CT09</t>
         </is>
       </c>
-      <c r="B14" s="401" t="n"/>
-      <c r="C14" s="401" t="n"/>
-      <c r="D14" s="401" t="n"/>
+      <c r="B14" s="385" t="n"/>
+      <c r="C14" s="399" t="n"/>
+      <c r="D14" s="385" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="401" t="n"/>
-      <c r="B15" s="401" t="n"/>
-      <c r="C15" s="401" t="n"/>
-      <c r="D15" s="401" t="n"/>
+      <c r="A15" s="385" t="n"/>
+      <c r="B15" s="399" t="n"/>
+      <c r="C15" s="385" t="n"/>
+      <c r="D15" s="399" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>HEX: #6B849D</t>
+          <t>HEX: #6B849D80</t>
         </is>
       </c>
       <c r="B16" s="15" t="n"/>
@@ -10972,7 +10969,7 @@
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>RGB: 107, 132, 157</t>
+          <t>RGB: 107, 132, 157, 128</t>
         </is>
       </c>
       <c r="B17" s="15" t="n"/>
@@ -10990,12 +10987,11 @@
       <c r="D18" s="15" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="27">
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="A17:D17"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="P13:S13"/>
-    <mergeCell ref="P9:S10"/>
     <mergeCell ref="P12:S12"/>
     <mergeCell ref="K7:N7"/>
     <mergeCell ref="A13:D13"/>
@@ -11004,29 +11000,21 @@
     <mergeCell ref="F11:I11"/>
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="F6:I6"/>
-    <mergeCell ref="A14:D15"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="F7:I7"/>
-    <mergeCell ref="F9:I10"/>
-    <mergeCell ref="A4:D5"/>
     <mergeCell ref="F12:I12"/>
     <mergeCell ref="K11:N11"/>
     <mergeCell ref="A7:D7"/>
-    <mergeCell ref="K4:N5"/>
     <mergeCell ref="P6:S6"/>
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="P8:S8"/>
     <mergeCell ref="P11:S11"/>
     <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A9:D10"/>
     <mergeCell ref="F8:I8"/>
     <mergeCell ref="A12:D12"/>
-    <mergeCell ref="K9:N10"/>
-    <mergeCell ref="F4:I5"/>
     <mergeCell ref="K12:N12"/>
     <mergeCell ref="P7:S7"/>
     <mergeCell ref="K8:N8"/>
-    <mergeCell ref="P4:S5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>